<commit_message>
v0.15.22.02: write the JANUS sheet the lab actually uses, eight columns with named plates
</commit_message>
<xml_diff>
--- a/src-tauri/samples/kuro/dmpR_sample_20260519/janus.xlsx
+++ b/src-tauri/samples/kuro/dmpR_sample_20260519/janus.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="layout" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="primer_mapping file" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="layout" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="primer_mapping file" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -939,6 +939,257 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Reverse primer usage</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>Source Well</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>Primer Name</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>Shared By (reactions)</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>Volume Per Reaction (µL)</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Total Transfer Volume (µL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Q232A_R</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Y233A_R</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>E335A_R</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>K200A_R</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>F203A_R</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>D227A_R</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>G237A_R</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>P240A_R</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Y155A_R</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>C175A_R</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Total Transfer Volume excludes instrument dead volume. Fill each source well with this total plus the dead volume of the labware in use.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -950,18 +1201,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -977,35 +1227,30 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Asp. Rack</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Asp. Posi</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Dsp. Rack</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Asp. Rack</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Asp. Posi</t>
-        </is>
-      </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Dsp. Rack</t>
+          <t>Dsp. Posi</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Dsp. Posi</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>volume</t>
         </is>
@@ -1014,7 +1259,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Q232A-fw</t>
+          <t>Q232A-F</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1022,38 +1267,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
-        <v>1</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
+      <c r="H2" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Y233A-fw</t>
+          <t>Y233A-F</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1061,38 +1305,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1</v>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
+      <c r="H3" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E335A-fw</t>
+          <t>E335A-F</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1100,38 +1343,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="C4" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="n">
-        <v>1</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
+      <c r="H4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>K200A-fw</t>
+          <t>K200A-F</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1139,38 +1381,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+      <c r="C5" t="n">
         <v>4</v>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
+      <c r="H5" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>F203A-fw</t>
+          <t>F203A-F</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1178,38 +1419,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+      <c r="C6" t="n">
         <v>5</v>
       </c>
-      <c r="E6" t="n">
-        <v>1</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>E1</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
+      <c r="H6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>D227A-fw</t>
+          <t>D227A-F</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1217,38 +1457,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
+      <c r="C7" t="n">
         <v>6</v>
       </c>
-      <c r="E7" t="n">
-        <v>1</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
+      <c r="H7" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>G237A-fw</t>
+          <t>G237A-F</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1256,38 +1495,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
+      <c r="C8" t="n">
         <v>7</v>
       </c>
-      <c r="E8" t="n">
-        <v>1</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>G1</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
+      <c r="H8" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P240A-fw</t>
+          <t>P240A-F</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1295,38 +1533,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
+      <c r="C9" t="n">
         <v>8</v>
       </c>
-      <c r="E9" t="n">
-        <v>1</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
+      <c r="H9" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Y155A-fw</t>
+          <t>Y155A-F</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1334,38 +1571,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
+      <c r="C10" t="n">
         <v>9</v>
       </c>
-      <c r="E10" t="n">
-        <v>1</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>2</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
+      <c r="H10" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C175A-fw</t>
+          <t>C175A-F</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1373,38 +1609,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
+      <c r="C11" t="n">
         <v>10</v>
       </c>
-      <c r="E11" t="n">
-        <v>1</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="G11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
+      <c r="H11" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Q232A-rv</t>
+          <t>Q232A-R</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1412,38 +1647,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
+      <c r="C12" t="n">
         <v>11</v>
       </c>
-      <c r="E12" t="n">
-        <v>2</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="G12" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
+      <c r="H12" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Y233A-rv</t>
+          <t>Y233A-R</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1451,38 +1685,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
+      <c r="C13" t="n">
         <v>12</v>
       </c>
-      <c r="E13" t="n">
-        <v>2</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="G13" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
+      <c r="H13" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>E335A-rv</t>
+          <t>E335A-R</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1490,38 +1723,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
+      <c r="C14" t="n">
         <v>13</v>
       </c>
-      <c r="E14" t="n">
-        <v>2</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="G14" t="n">
-        <v>2</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
+      <c r="H14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>K200A-rv</t>
+          <t>K200A-R</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1529,38 +1761,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
+      <c r="C15" t="n">
         <v>14</v>
       </c>
-      <c r="E15" t="n">
-        <v>2</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="G15" t="n">
-        <v>2</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
+      <c r="H15" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>F203A-rv</t>
+          <t>F203A-R</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1568,38 +1799,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
+      <c r="C16" t="n">
         <v>15</v>
       </c>
-      <c r="E16" t="n">
-        <v>2</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
           <t>E1</t>
         </is>
       </c>
-      <c r="G16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
+      <c r="H16" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>D227A-rv</t>
+          <t>D227A-R</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1607,38 +1837,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
+      <c r="C17" t="n">
         <v>16</v>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="G17" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
+      <c r="H17" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>G237A-rv</t>
+          <t>G237A-R</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1646,38 +1875,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
+      <c r="C18" t="n">
         <v>17</v>
       </c>
-      <c r="E18" t="n">
-        <v>2</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>G1</t>
         </is>
       </c>
-      <c r="G18" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
+      <c r="H18" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P240A-rv</t>
+          <t>P240A-R</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1685,38 +1913,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
+      <c r="C19" t="n">
         <v>18</v>
       </c>
-      <c r="E19" t="n">
-        <v>2</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="G19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
+      <c r="H19" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Y155A-rv</t>
+          <t>Y155A-R</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1724,38 +1951,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+      <c r="C20" t="n">
         <v>19</v>
       </c>
-      <c r="E20" t="n">
-        <v>2</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="G20" t="n">
-        <v>2</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
+      <c r="H20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C175A-rv</t>
+          <t>C175A-R</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1763,31 +1989,30 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
+      <c r="C21" t="n">
         <v>20</v>
       </c>
-      <c r="E21" t="n">
-        <v>2</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="G21" t="n">
-        <v>2</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
+      <c r="H21" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.16.1: give the robot the sheet the lab uses, and let the review screen explain itself
Merged from #267. Full detail in the PR description and CHANGELOG v0.16.1.
</commit_message>
<xml_diff>
--- a/src-tauri/samples/kuro/dmpR_sample_20260519/janus.xlsx
+++ b/src-tauri/samples/kuro/dmpR_sample_20260519/janus.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="layout" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="primer_mapping file" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="layout" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="primer_mapping file" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -939,6 +939,257 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Reverse primer usage</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>Source Well</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>Primer Name</t>
+        </is>
+      </c>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>Shared By (reactions)</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>Volume Per Reaction (µL)</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>Total Transfer Volume (µL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Q232A_R</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Y233A_R</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>E335A_R</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>K200A_R</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>F203A_R</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>D227A_R</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>G237A_R</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>P240A_R</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Y155A_R</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>C175A_R</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Total Transfer Volume excludes instrument dead volume. Fill each source well with this total plus the dead volume of the labware in use.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -950,18 +1201,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="4" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -977,35 +1227,30 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Asp. Rack</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Asp. Posi</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Dsp. Rack</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Asp. Rack</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Asp. Posi</t>
-        </is>
-      </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Dsp. Rack</t>
+          <t>Dsp. Posi</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Dsp. Posi</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>volume</t>
         </is>
@@ -1014,7 +1259,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Q232A-fw</t>
+          <t>Q232A-F</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1022,38 +1267,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="C2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="n">
-        <v>1</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="I2" t="n">
+      <c r="H2" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Y233A-fw</t>
+          <t>Y233A-F</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1061,38 +1305,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1</v>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="I3" t="n">
+      <c r="H3" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E335A-fw</t>
+          <t>E335A-F</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1100,38 +1343,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
+      <c r="C4" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="n">
-        <v>1</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
+      <c r="H4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>K200A-fw</t>
+          <t>K200A-F</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1139,38 +1381,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
+      <c r="C5" t="n">
         <v>4</v>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
+      <c r="H5" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>F203A-fw</t>
+          <t>F203A-F</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1178,38 +1419,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
+      <c r="C6" t="n">
         <v>5</v>
       </c>
-      <c r="E6" t="n">
-        <v>1</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>E1</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
+      <c r="H6" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>D227A-fw</t>
+          <t>D227A-F</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1217,38 +1457,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
+      <c r="C7" t="n">
         <v>6</v>
       </c>
-      <c r="E7" t="n">
-        <v>1</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
+      <c r="H7" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>G237A-fw</t>
+          <t>G237A-F</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1256,38 +1495,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
+      <c r="C8" t="n">
         <v>7</v>
       </c>
-      <c r="E8" t="n">
-        <v>1</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>G1</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>2</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
+      <c r="H8" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>P240A-fw</t>
+          <t>P240A-F</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1295,38 +1533,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
+      <c r="C9" t="n">
         <v>8</v>
       </c>
-      <c r="E9" t="n">
-        <v>1</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
+      <c r="H9" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Y155A-fw</t>
+          <t>Y155A-F</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1334,38 +1571,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
+      <c r="C10" t="n">
         <v>9</v>
       </c>
-      <c r="E10" t="n">
-        <v>1</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>2</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="I10" t="n">
+      <c r="H10" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C175A-fw</t>
+          <t>C175A-F</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1373,38 +1609,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
+      <c r="C11" t="n">
         <v>10</v>
       </c>
-      <c r="E11" t="n">
-        <v>1</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fw plate</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="G11" t="n">
-        <v>2</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
+      <c r="H11" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Q232A-rv</t>
+          <t>Q232A-R</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1412,38 +1647,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
+      <c r="C12" t="n">
         <v>11</v>
       </c>
-      <c r="E12" t="n">
-        <v>2</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="G12" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
+      <c r="H12" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Y233A-rv</t>
+          <t>Y233A-R</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1451,38 +1685,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
+      <c r="C13" t="n">
         <v>12</v>
       </c>
-      <c r="E13" t="n">
-        <v>2</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>B1</t>
         </is>
       </c>
-      <c r="G13" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
+      <c r="H13" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>E335A-rv</t>
+          <t>E335A-R</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1490,38 +1723,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
+      <c r="C14" t="n">
         <v>13</v>
       </c>
-      <c r="E14" t="n">
-        <v>2</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="G14" t="n">
-        <v>2</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="I14" t="n">
+      <c r="H14" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>K200A-rv</t>
+          <t>K200A-R</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1529,38 +1761,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
+      <c r="C15" t="n">
         <v>14</v>
       </c>
-      <c r="E15" t="n">
-        <v>2</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="G15" t="n">
-        <v>2</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
+      <c r="H15" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>F203A-rv</t>
+          <t>F203A-R</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1568,38 +1799,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
+      <c r="C16" t="n">
         <v>15</v>
       </c>
-      <c r="E16" t="n">
-        <v>2</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
           <t>E1</t>
         </is>
       </c>
-      <c r="G16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>E1</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
+      <c r="H16" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>D227A-rv</t>
+          <t>D227A-R</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1607,38 +1837,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
+      <c r="C17" t="n">
         <v>16</v>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>F1</t>
         </is>
       </c>
-      <c r="G17" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>F1</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
+      <c r="H17" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>G237A-rv</t>
+          <t>G237A-R</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1646,38 +1875,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
+      <c r="C18" t="n">
         <v>17</v>
       </c>
-      <c r="E18" t="n">
-        <v>2</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
           <t>G1</t>
         </is>
       </c>
-      <c r="G18" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>G1</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
+      <c r="H18" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>P240A-rv</t>
+          <t>P240A-R</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1685,38 +1913,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
+      <c r="C19" t="n">
         <v>18</v>
       </c>
-      <c r="E19" t="n">
-        <v>2</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="G19" t="n">
-        <v>2</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
+      <c r="H19" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Y155A-rv</t>
+          <t>Y155A-R</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1724,38 +1951,37 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+      <c r="C20" t="n">
         <v>19</v>
       </c>
-      <c r="E20" t="n">
-        <v>2</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="G20" t="n">
-        <v>2</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
+      <c r="H20" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C175A-rv</t>
+          <t>C175A-R</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1763,31 +1989,30 @@
           <t>primer</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Oligo 5pmol/ul</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
+      <c r="C21" t="n">
         <v>20</v>
       </c>
-      <c r="E21" t="n">
-        <v>2</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>rv plate</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
+          <t>PCR mixture plate</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
           <t>B2</t>
         </is>
       </c>
-      <c r="G21" t="n">
-        <v>2</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
+      <c r="H21" t="n">
         <v>2</v>
       </c>
     </row>

</xml_diff>